<commit_message>
feat(core): add number-to-word conversion and improve address display
This commit introduces the following changes:

Add a new function to convert numbers into Indian word standard.

Update address display in:

Print preview page
Invoice Excel download
Improve Excel export formatting:

Each project is now displayed on a new line within the same cell
Implement text wrapping
These changes improve the overall functionality and user experience
of the application.
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27830"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF26F80D-8DDB-4B23-BF97-C1A8C2A0CC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85CF836F-5F27-4874-835B-443274492FE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -14,6 +14,17 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Summary!$B$1:$P$66</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -131,12 +142,6 @@
     <t xml:space="preserve">TAN: </t>
   </si>
   <si>
-    <t xml:space="preserve">Plot No 104, 2nd Cross Street, </t>
-  </si>
-  <si>
-    <t>VGP Sea View Part - 1, Palavakkam,</t>
-  </si>
-  <si>
     <t>Chennai - 600 041</t>
   </si>
   <si>
@@ -230,6 +235,12 @@
   <si>
     <t>Purchase of renewable attributes for I-REC
 (20028.63 units at INR 51.68124 per unit)</t>
+  </si>
+  <si>
+    <t>F1 Plot, 3rd Street, Kuberan Nagar,</t>
+  </si>
+  <si>
+    <t>Extension,Madipakkam,</t>
   </si>
 </sst>
 </file>
@@ -582,7 +593,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -691,6 +702,36 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -698,9 +739,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -715,32 +753,8 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1053,41 +1067,41 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S66"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="4.5546875" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="4.54296875" customWidth="1"/>
+    <col min="3" max="3" width="10.36328125" customWidth="1"/>
+    <col min="6" max="6" width="12.08984375" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" customWidth="1"/>
-    <col min="11" max="11" width="13.109375" customWidth="1"/>
-    <col min="12" max="12" width="8.5546875" customWidth="1"/>
-    <col min="13" max="13" width="14.88671875" customWidth="1"/>
-    <col min="14" max="14" width="8.5546875" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" customWidth="1"/>
+    <col min="11" max="11" width="13.08984375" customWidth="1"/>
+    <col min="12" max="12" width="8.54296875" customWidth="1"/>
+    <col min="13" max="13" width="14.90625" customWidth="1"/>
+    <col min="14" max="14" width="8.54296875" customWidth="1"/>
     <col min="15" max="15" width="15" customWidth="1"/>
-    <col min="16" max="16" width="10.33203125" customWidth="1"/>
-    <col min="18" max="18" width="11.33203125" customWidth="1"/>
+    <col min="16" max="16" width="10.36328125" customWidth="1"/>
+    <col min="18" max="18" width="11.36328125" customWidth="1"/>
     <col min="19" max="19" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
       <c r="A1" s="1"/>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
@@ -1138,7 +1152,7 @@
       <c r="A4" s="2"/>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1146,10 +1160,10 @@
       <c r="G4" s="9"/>
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
-      <c r="J4" s="59"/>
-      <c r="K4" s="59"/>
-      <c r="L4" s="59"/>
-      <c r="M4" s="59"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="69"/>
+      <c r="L4" s="69"/>
+      <c r="M4" s="69"/>
       <c r="N4" s="9"/>
       <c r="O4" s="9"/>
       <c r="P4" s="10"/>
@@ -1161,7 +1175,7 @@
       <c r="A5" s="2"/>
       <c r="B5" s="7"/>
       <c r="C5" s="11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -1169,10 +1183,10 @@
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-      <c r="L5" s="59"/>
-      <c r="M5" s="59"/>
+      <c r="J5" s="69"/>
+      <c r="K5" s="69"/>
+      <c r="L5" s="69"/>
+      <c r="M5" s="69"/>
       <c r="N5" s="9"/>
       <c r="O5" s="9"/>
       <c r="P5" s="10"/>
@@ -1184,7 +1198,7 @@
       <c r="A6" s="2"/>
       <c r="B6" s="7"/>
       <c r="C6" s="11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -1203,7 +1217,7 @@
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
     </row>
-    <row r="7" spans="1:19" ht="28.2" thickBot="1">
+    <row r="7" spans="1:19" ht="28" thickBot="1">
       <c r="A7" s="2"/>
       <c r="B7" s="7"/>
       <c r="C7" s="13" t="s">
@@ -1213,11 +1227,11 @@
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
-      <c r="H7" s="65" t="s">
-        <v>45</v>
-      </c>
-      <c r="I7" s="65"/>
-      <c r="J7" s="65"/>
+      <c r="H7" s="74" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="74"/>
+      <c r="J7" s="74"/>
       <c r="K7" s="14"/>
       <c r="L7" s="14"/>
       <c r="M7" s="14"/>
@@ -1263,7 +1277,7 @@
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
       <c r="K9" s="12" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L9" s="12"/>
       <c r="M9" s="17"/>
@@ -1288,7 +1302,7 @@
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
       <c r="K10" s="12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="L10" s="12"/>
       <c r="M10" s="12"/>
@@ -1349,7 +1363,7 @@
       <c r="A13" s="2"/>
       <c r="B13" s="7"/>
       <c r="C13" s="9" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -1359,7 +1373,7 @@
       <c r="I13" s="9"/>
       <c r="J13" s="9"/>
       <c r="K13" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L13" s="9"/>
       <c r="M13" s="9"/>
@@ -1374,7 +1388,7 @@
       <c r="A14" s="2"/>
       <c r="B14" s="7"/>
       <c r="C14" s="9" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -1397,7 +1411,7 @@
       <c r="A15" s="2"/>
       <c r="B15" s="7"/>
       <c r="C15" s="19" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -1440,7 +1454,7 @@
     <row r="17" spans="2:19" ht="18">
       <c r="B17" s="7"/>
       <c r="C17" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
@@ -1485,14 +1499,14 @@
     <row r="19" spans="2:19" ht="18">
       <c r="B19" s="7"/>
       <c r="C19" s="11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
       <c r="G19" s="54"/>
       <c r="H19" s="11" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I19" s="11"/>
       <c r="J19" s="9"/>
@@ -1511,14 +1525,14 @@
     <row r="20" spans="2:19" ht="18">
       <c r="B20" s="7"/>
       <c r="C20" s="55" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
       <c r="H20" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I20" s="9"/>
       <c r="J20" s="9"/>
@@ -1553,13 +1567,13 @@
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
     </row>
-    <row r="22" spans="2:19" ht="34.200000000000003" customHeight="1">
+    <row r="22" spans="2:19" ht="34.25" customHeight="1">
       <c r="B22" s="7"/>
-      <c r="C22" s="64"/>
-      <c r="D22" s="64"/>
-      <c r="E22" s="64"/>
-      <c r="F22" s="64"/>
-      <c r="G22" s="64"/>
+      <c r="C22" s="73"/>
+      <c r="D22" s="73"/>
+      <c r="E22" s="73"/>
+      <c r="F22" s="73"/>
+      <c r="G22" s="73"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="9"/>
@@ -1616,11 +1630,11 @@
     <row r="25" spans="2:19" ht="18">
       <c r="B25" s="7"/>
       <c r="C25" s="11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -1642,11 +1656,11 @@
     <row r="26" spans="2:19" ht="18">
       <c r="B26" s="7"/>
       <c r="C26" s="11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -1687,33 +1701,33 @@
     </row>
     <row r="28" spans="2:19" ht="21" customHeight="1">
       <c r="B28" s="7"/>
-      <c r="C28" s="60" t="s">
+      <c r="C28" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="D28" s="60"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="61" t="s">
+      <c r="D28" s="64"/>
+      <c r="E28" s="64"/>
+      <c r="F28" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="G28" s="61" t="s">
+      <c r="G28" s="70" t="s">
         <v>9</v>
       </c>
-      <c r="H28" s="60" t="s">
+      <c r="H28" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="I28" s="60"/>
-      <c r="J28" s="60" t="s">
+      <c r="I28" s="64"/>
+      <c r="J28" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="K28" s="60"/>
-      <c r="L28" s="60" t="s">
+      <c r="K28" s="64"/>
+      <c r="L28" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="M28" s="62"/>
-      <c r="N28" s="62" t="s">
+      <c r="M28" s="71"/>
+      <c r="N28" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="O28" s="63"/>
+      <c r="O28" s="72"/>
       <c r="P28" s="10"/>
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
@@ -1721,11 +1735,11 @@
     </row>
     <row r="29" spans="2:19" ht="18">
       <c r="B29" s="7"/>
-      <c r="C29" s="60"/>
-      <c r="D29" s="60"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="61"/>
-      <c r="G29" s="61"/>
+      <c r="C29" s="64"/>
+      <c r="D29" s="64"/>
+      <c r="E29" s="64"/>
+      <c r="F29" s="70"/>
+      <c r="G29" s="70"/>
       <c r="H29" s="22" t="s">
         <v>14</v>
       </c>
@@ -1777,13 +1791,13 @@
     </row>
     <row r="31" spans="2:19" ht="99.9" customHeight="1">
       <c r="B31" s="7"/>
-      <c r="C31" s="69" t="s">
-        <v>54</v>
-      </c>
-      <c r="D31" s="70"/>
-      <c r="E31" s="71"/>
+      <c r="C31" s="61" t="s">
+        <v>52</v>
+      </c>
+      <c r="D31" s="62"/>
+      <c r="E31" s="63"/>
       <c r="F31" s="29" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G31" s="30">
         <f>20028.63*51.68124</f>
@@ -1920,12 +1934,12 @@
     </row>
     <row r="37" spans="2:19" ht="18">
       <c r="B37" s="7"/>
-      <c r="C37" s="60" t="s">
+      <c r="C37" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="D37" s="60"/>
-      <c r="E37" s="60"/>
-      <c r="F37" s="60"/>
+      <c r="D37" s="64"/>
+      <c r="E37" s="64"/>
+      <c r="F37" s="64"/>
       <c r="G37" s="39">
         <f>SUM(G30:G36)</f>
         <v>1035104.4339012001</v>
@@ -2008,15 +2022,15 @@
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
       <c r="F40" s="11"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="68"/>
-      <c r="I40" s="68"/>
-      <c r="J40" s="68"/>
-      <c r="K40" s="68"/>
-      <c r="L40" s="68"/>
-      <c r="M40" s="68"/>
-      <c r="N40" s="68"/>
-      <c r="O40" s="68"/>
+      <c r="G40" s="75"/>
+      <c r="H40" s="75"/>
+      <c r="I40" s="75"/>
+      <c r="J40" s="75"/>
+      <c r="K40" s="75"/>
+      <c r="L40" s="75"/>
+      <c r="M40" s="75"/>
+      <c r="N40" s="75"/>
+      <c r="O40" s="75"/>
       <c r="P40" s="10"/>
       <c r="Q40" s="2"/>
       <c r="R40" s="2"/>
@@ -2051,14 +2065,14 @@
       <c r="E42" s="9"/>
       <c r="F42" s="11"/>
       <c r="G42" s="9"/>
-      <c r="H42" s="72"/>
-      <c r="I42" s="73"/>
-      <c r="J42" s="72"/>
-      <c r="K42" s="73"/>
-      <c r="L42" s="72"/>
-      <c r="M42" s="74"/>
-      <c r="N42" s="72"/>
-      <c r="O42" s="73"/>
+      <c r="H42" s="65"/>
+      <c r="I42" s="66"/>
+      <c r="J42" s="65"/>
+      <c r="K42" s="66"/>
+      <c r="L42" s="65"/>
+      <c r="M42" s="67"/>
+      <c r="N42" s="65"/>
+      <c r="O42" s="66"/>
       <c r="P42" s="10"/>
       <c r="Q42" s="2"/>
       <c r="R42" s="2"/>
@@ -2118,7 +2132,7 @@
       <c r="J45" s="9"/>
       <c r="K45" s="9"/>
       <c r="L45" s="45" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M45" s="45"/>
       <c r="N45" s="9"/>
@@ -2131,7 +2145,7 @@
     <row r="46" spans="2:19" ht="18">
       <c r="B46" s="7"/>
       <c r="C46" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
@@ -2153,7 +2167,7 @@
     <row r="47" spans="2:19" ht="18">
       <c r="B47" s="7"/>
       <c r="C47" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
@@ -2175,7 +2189,7 @@
     <row r="48" spans="2:19" ht="18">
       <c r="B48" s="7"/>
       <c r="C48" s="9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
@@ -2196,7 +2210,7 @@
     <row r="49" spans="2:19" ht="18">
       <c r="B49" s="7"/>
       <c r="C49" s="9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
@@ -2217,7 +2231,7 @@
     <row r="50" spans="2:19" ht="18">
       <c r="B50" s="7"/>
       <c r="C50" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
@@ -2296,59 +2310,59 @@
     </row>
     <row r="54" spans="2:19" ht="15" customHeight="1">
       <c r="B54" s="7"/>
-      <c r="C54" s="66" t="s">
-        <v>38</v>
-      </c>
-      <c r="D54" s="66"/>
-      <c r="E54" s="66"/>
-      <c r="F54" s="66"/>
-      <c r="G54" s="66"/>
-      <c r="H54" s="66"/>
-      <c r="I54" s="66"/>
-      <c r="J54" s="66"/>
-      <c r="K54" s="66"/>
-      <c r="L54" s="66"/>
-      <c r="M54" s="66"/>
-      <c r="N54" s="66"/>
-      <c r="O54" s="66"/>
+      <c r="C54" s="58" t="s">
+        <v>36</v>
+      </c>
+      <c r="D54" s="58"/>
+      <c r="E54" s="58"/>
+      <c r="F54" s="58"/>
+      <c r="G54" s="58"/>
+      <c r="H54" s="58"/>
+      <c r="I54" s="58"/>
+      <c r="J54" s="58"/>
+      <c r="K54" s="58"/>
+      <c r="L54" s="58"/>
+      <c r="M54" s="58"/>
+      <c r="N54" s="58"/>
+      <c r="O54" s="58"/>
       <c r="P54" s="10"/>
       <c r="Q54" s="2"/>
       <c r="R54" s="2"/>
     </row>
     <row r="55" spans="2:19" ht="18">
       <c r="B55" s="7"/>
-      <c r="C55" s="66"/>
-      <c r="D55" s="66"/>
-      <c r="E55" s="66"/>
-      <c r="F55" s="66"/>
-      <c r="G55" s="66"/>
-      <c r="H55" s="66"/>
-      <c r="I55" s="66"/>
-      <c r="J55" s="66"/>
-      <c r="K55" s="66"/>
-      <c r="L55" s="66"/>
-      <c r="M55" s="66"/>
-      <c r="N55" s="66"/>
-      <c r="O55" s="66"/>
+      <c r="C55" s="58"/>
+      <c r="D55" s="58"/>
+      <c r="E55" s="58"/>
+      <c r="F55" s="58"/>
+      <c r="G55" s="58"/>
+      <c r="H55" s="58"/>
+      <c r="I55" s="58"/>
+      <c r="J55" s="58"/>
+      <c r="K55" s="58"/>
+      <c r="L55" s="58"/>
+      <c r="M55" s="58"/>
+      <c r="N55" s="58"/>
+      <c r="O55" s="58"/>
       <c r="P55" s="10"/>
       <c r="Q55" s="2"/>
       <c r="R55" s="2"/>
     </row>
     <row r="56" spans="2:19" ht="18">
       <c r="B56" s="7"/>
-      <c r="C56" s="66"/>
-      <c r="D56" s="66"/>
-      <c r="E56" s="66"/>
-      <c r="F56" s="66"/>
-      <c r="G56" s="66"/>
-      <c r="H56" s="66"/>
-      <c r="I56" s="66"/>
-      <c r="J56" s="66"/>
-      <c r="K56" s="66"/>
-      <c r="L56" s="66"/>
-      <c r="M56" s="66"/>
-      <c r="N56" s="66"/>
-      <c r="O56" s="66"/>
+      <c r="C56" s="58"/>
+      <c r="D56" s="58"/>
+      <c r="E56" s="58"/>
+      <c r="F56" s="58"/>
+      <c r="G56" s="58"/>
+      <c r="H56" s="58"/>
+      <c r="I56" s="58"/>
+      <c r="J56" s="58"/>
+      <c r="K56" s="58"/>
+      <c r="L56" s="58"/>
+      <c r="M56" s="58"/>
+      <c r="N56" s="58"/>
+      <c r="O56" s="58"/>
       <c r="P56" s="10"/>
       <c r="Q56" s="2"/>
       <c r="R56" s="2"/>
@@ -2356,19 +2370,19 @@
     </row>
     <row r="57" spans="2:19" ht="18">
       <c r="B57" s="7"/>
-      <c r="C57" s="66"/>
-      <c r="D57" s="66"/>
-      <c r="E57" s="66"/>
-      <c r="F57" s="66"/>
-      <c r="G57" s="66"/>
-      <c r="H57" s="66"/>
-      <c r="I57" s="66"/>
-      <c r="J57" s="66"/>
-      <c r="K57" s="66"/>
-      <c r="L57" s="66"/>
-      <c r="M57" s="66"/>
-      <c r="N57" s="66"/>
-      <c r="O57" s="66"/>
+      <c r="C57" s="58"/>
+      <c r="D57" s="58"/>
+      <c r="E57" s="58"/>
+      <c r="F57" s="58"/>
+      <c r="G57" s="58"/>
+      <c r="H57" s="58"/>
+      <c r="I57" s="58"/>
+      <c r="J57" s="58"/>
+      <c r="K57" s="58"/>
+      <c r="L57" s="58"/>
+      <c r="M57" s="58"/>
+      <c r="N57" s="58"/>
+      <c r="O57" s="58"/>
       <c r="P57" s="10"/>
       <c r="Q57" s="2"/>
       <c r="R57" s="2"/>
@@ -2376,19 +2390,19 @@
     </row>
     <row r="58" spans="2:19" ht="23.25" customHeight="1">
       <c r="B58" s="7"/>
-      <c r="C58" s="66"/>
-      <c r="D58" s="66"/>
-      <c r="E58" s="66"/>
-      <c r="F58" s="66"/>
-      <c r="G58" s="66"/>
-      <c r="H58" s="66"/>
-      <c r="I58" s="66"/>
-      <c r="J58" s="66"/>
-      <c r="K58" s="66"/>
-      <c r="L58" s="66"/>
-      <c r="M58" s="66"/>
-      <c r="N58" s="66"/>
-      <c r="O58" s="66"/>
+      <c r="C58" s="58"/>
+      <c r="D58" s="58"/>
+      <c r="E58" s="58"/>
+      <c r="F58" s="58"/>
+      <c r="G58" s="58"/>
+      <c r="H58" s="58"/>
+      <c r="I58" s="58"/>
+      <c r="J58" s="58"/>
+      <c r="K58" s="58"/>
+      <c r="L58" s="58"/>
+      <c r="M58" s="58"/>
+      <c r="N58" s="58"/>
+      <c r="O58" s="58"/>
       <c r="P58" s="10"/>
       <c r="Q58" s="2"/>
       <c r="R58" s="2"/>
@@ -2396,19 +2410,19 @@
     </row>
     <row r="59" spans="2:19" ht="23.25" customHeight="1">
       <c r="B59" s="7"/>
-      <c r="C59" s="66"/>
-      <c r="D59" s="66"/>
-      <c r="E59" s="66"/>
-      <c r="F59" s="66"/>
-      <c r="G59" s="66"/>
-      <c r="H59" s="66"/>
-      <c r="I59" s="66"/>
-      <c r="J59" s="66"/>
-      <c r="K59" s="66"/>
-      <c r="L59" s="66"/>
-      <c r="M59" s="66"/>
-      <c r="N59" s="66"/>
-      <c r="O59" s="66"/>
+      <c r="C59" s="58"/>
+      <c r="D59" s="58"/>
+      <c r="E59" s="58"/>
+      <c r="F59" s="58"/>
+      <c r="G59" s="58"/>
+      <c r="H59" s="58"/>
+      <c r="I59" s="58"/>
+      <c r="J59" s="58"/>
+      <c r="K59" s="58"/>
+      <c r="L59" s="58"/>
+      <c r="M59" s="58"/>
+      <c r="N59" s="58"/>
+      <c r="O59" s="58"/>
       <c r="P59" s="10"/>
       <c r="Q59" s="2"/>
       <c r="R59" s="2"/>
@@ -2416,19 +2430,19 @@
     </row>
     <row r="60" spans="2:19" ht="23.25" customHeight="1">
       <c r="B60" s="7"/>
-      <c r="C60" s="66"/>
-      <c r="D60" s="66"/>
-      <c r="E60" s="66"/>
-      <c r="F60" s="66"/>
-      <c r="G60" s="66"/>
-      <c r="H60" s="66"/>
-      <c r="I60" s="66"/>
-      <c r="J60" s="66"/>
-      <c r="K60" s="66"/>
-      <c r="L60" s="66"/>
-      <c r="M60" s="66"/>
-      <c r="N60" s="66"/>
-      <c r="O60" s="66"/>
+      <c r="C60" s="58"/>
+      <c r="D60" s="58"/>
+      <c r="E60" s="58"/>
+      <c r="F60" s="58"/>
+      <c r="G60" s="58"/>
+      <c r="H60" s="58"/>
+      <c r="I60" s="58"/>
+      <c r="J60" s="58"/>
+      <c r="K60" s="58"/>
+      <c r="L60" s="58"/>
+      <c r="M60" s="58"/>
+      <c r="N60" s="58"/>
+      <c r="O60" s="58"/>
       <c r="P60" s="10"/>
       <c r="Q60" s="2"/>
       <c r="R60" s="2"/>
@@ -2436,19 +2450,19 @@
     </row>
     <row r="61" spans="2:19" ht="23.25" customHeight="1">
       <c r="B61" s="7"/>
-      <c r="C61" s="66"/>
-      <c r="D61" s="66"/>
-      <c r="E61" s="66"/>
-      <c r="F61" s="66"/>
-      <c r="G61" s="66"/>
-      <c r="H61" s="66"/>
-      <c r="I61" s="66"/>
-      <c r="J61" s="66"/>
-      <c r="K61" s="66"/>
-      <c r="L61" s="66"/>
-      <c r="M61" s="66"/>
-      <c r="N61" s="66"/>
-      <c r="O61" s="66"/>
+      <c r="C61" s="58"/>
+      <c r="D61" s="58"/>
+      <c r="E61" s="58"/>
+      <c r="F61" s="58"/>
+      <c r="G61" s="58"/>
+      <c r="H61" s="58"/>
+      <c r="I61" s="58"/>
+      <c r="J61" s="58"/>
+      <c r="K61" s="58"/>
+      <c r="L61" s="58"/>
+      <c r="M61" s="58"/>
+      <c r="N61" s="58"/>
+      <c r="O61" s="58"/>
       <c r="P61" s="10"/>
       <c r="Q61" s="2"/>
       <c r="R61" s="2"/>
@@ -2496,21 +2510,21 @@
     </row>
     <row r="64" spans="2:19" ht="18" hidden="1">
       <c r="B64" s="7"/>
-      <c r="C64" s="67" t="s">
+      <c r="C64" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="D64" s="67"/>
-      <c r="E64" s="67"/>
-      <c r="F64" s="67"/>
-      <c r="G64" s="67"/>
-      <c r="H64" s="67"/>
-      <c r="I64" s="67"/>
-      <c r="J64" s="67"/>
-      <c r="K64" s="67"/>
-      <c r="L64" s="67"/>
-      <c r="M64" s="67"/>
-      <c r="N64" s="67"/>
-      <c r="O64" s="67"/>
+      <c r="D64" s="59"/>
+      <c r="E64" s="59"/>
+      <c r="F64" s="59"/>
+      <c r="G64" s="59"/>
+      <c r="H64" s="59"/>
+      <c r="I64" s="59"/>
+      <c r="J64" s="59"/>
+      <c r="K64" s="59"/>
+      <c r="L64" s="59"/>
+      <c r="M64" s="59"/>
+      <c r="N64" s="59"/>
+      <c r="O64" s="59"/>
       <c r="P64" s="10"/>
       <c r="Q64" s="2"/>
       <c r="R64" s="2"/>
@@ -2518,27 +2532,27 @@
     </row>
     <row r="65" spans="2:19" ht="18" hidden="1">
       <c r="B65" s="7"/>
-      <c r="C65" s="68" t="s">
+      <c r="C65" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="D65" s="68"/>
-      <c r="E65" s="68"/>
-      <c r="F65" s="68"/>
-      <c r="G65" s="68"/>
-      <c r="H65" s="68"/>
-      <c r="I65" s="68"/>
-      <c r="J65" s="68"/>
-      <c r="K65" s="68"/>
-      <c r="L65" s="68"/>
-      <c r="M65" s="68"/>
-      <c r="N65" s="68"/>
-      <c r="O65" s="68"/>
+      <c r="D65" s="60"/>
+      <c r="E65" s="60"/>
+      <c r="F65" s="60"/>
+      <c r="G65" s="60"/>
+      <c r="H65" s="60"/>
+      <c r="I65" s="60"/>
+      <c r="J65" s="60"/>
+      <c r="K65" s="60"/>
+      <c r="L65" s="60"/>
+      <c r="M65" s="60"/>
+      <c r="N65" s="60"/>
+      <c r="O65" s="60"/>
       <c r="P65" s="10"/>
       <c r="Q65" s="2"/>
       <c r="R65" s="2"/>
       <c r="S65" s="2"/>
     </row>
-    <row r="66" spans="2:19" ht="18.600000000000001" thickBot="1">
+    <row r="66" spans="2:19" ht="18.5" thickBot="1">
       <c r="B66" s="52"/>
       <c r="C66" s="15"/>
       <c r="D66" s="15"/>
@@ -2560,16 +2574,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C54:O61"/>
-    <mergeCell ref="C64:O64"/>
-    <mergeCell ref="C65:O65"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="H40:O40"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="N42:O42"/>
     <mergeCell ref="B1:P1"/>
     <mergeCell ref="J4:M4"/>
     <mergeCell ref="J5:M5"/>
@@ -2582,6 +2586,16 @@
     <mergeCell ref="N28:O28"/>
     <mergeCell ref="C22:G22"/>
     <mergeCell ref="H7:J7"/>
+    <mergeCell ref="C54:O61"/>
+    <mergeCell ref="C64:O64"/>
+    <mergeCell ref="C65:O65"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="G40:O40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="55" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix(forms): update pincode and terminology in invoice template
Changed the pincode and updated the terminology in the invoice template. This ensures that the invoice contains accurate and current information, enhancing both clarity and correctness.
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85CF836F-5F27-4874-835B-443274492FE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46B13ECE-B435-499F-81DD-13ECCB667976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -142,9 +142,6 @@
     <t xml:space="preserve">TAN: </t>
   </si>
   <si>
-    <t>Chennai - 600 041</t>
-  </si>
-  <si>
     <t>GSTIN: 33ABHCS3747D1ZG</t>
   </si>
   <si>
@@ -233,14 +230,17 @@
     <t>24 MW Wind Power Project in Kayathar, HTSC No.279-290</t>
   </si>
   <si>
-    <t>Purchase of renewable attributes for I-REC
+    <t>F1 Plot, 3rd Street, Kuberan Nagar,</t>
+  </si>
+  <si>
+    <t>Extension,Madipakkam,</t>
+  </si>
+  <si>
+    <t>Chennai - 600 091</t>
+  </si>
+  <si>
+    <t>Sale of renewable attributes for I-REC
 (20028.63 units at INR 51.68124 per unit)</t>
-  </si>
-  <si>
-    <t>F1 Plot, 3rd Street, Kuberan Nagar,</t>
-  </si>
-  <si>
-    <t>Extension,Madipakkam,</t>
   </si>
 </sst>
 </file>
@@ -702,6 +702,30 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -720,9 +744,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -731,27 +752,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1087,21 +1087,21 @@
   <sheetData>
     <row r="1" spans="1:19">
       <c r="A1" s="1"/>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
+      <c r="J1" s="58"/>
+      <c r="K1" s="58"/>
+      <c r="L1" s="58"/>
+      <c r="M1" s="58"/>
+      <c r="N1" s="58"/>
+      <c r="O1" s="58"/>
+      <c r="P1" s="58"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
       <c r="S1" s="2"/>
@@ -1152,7 +1152,7 @@
       <c r="A4" s="2"/>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1160,10 +1160,10 @@
       <c r="G4" s="9"/>
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
-      <c r="J4" s="69"/>
-      <c r="K4" s="69"/>
-      <c r="L4" s="69"/>
-      <c r="M4" s="69"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
       <c r="N4" s="9"/>
       <c r="O4" s="9"/>
       <c r="P4" s="10"/>
@@ -1175,7 +1175,7 @@
       <c r="A5" s="2"/>
       <c r="B5" s="7"/>
       <c r="C5" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -1183,10 +1183,10 @@
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
-      <c r="J5" s="69"/>
-      <c r="K5" s="69"/>
-      <c r="L5" s="69"/>
-      <c r="M5" s="69"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="59"/>
+      <c r="L5" s="59"/>
+      <c r="M5" s="59"/>
       <c r="N5" s="9"/>
       <c r="O5" s="9"/>
       <c r="P5" s="10"/>
@@ -1198,7 +1198,7 @@
       <c r="A6" s="2"/>
       <c r="B6" s="7"/>
       <c r="C6" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -1227,11 +1227,11 @@
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
       <c r="G7" s="14"/>
-      <c r="H7" s="74" t="s">
-        <v>43</v>
-      </c>
-      <c r="I7" s="74"/>
-      <c r="J7" s="74"/>
+      <c r="H7" s="65" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" s="65"/>
+      <c r="J7" s="65"/>
       <c r="K7" s="14"/>
       <c r="L7" s="14"/>
       <c r="M7" s="14"/>
@@ -1277,7 +1277,7 @@
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
       <c r="K9" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L9" s="12"/>
       <c r="M9" s="17"/>
@@ -1302,7 +1302,7 @@
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
       <c r="K10" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L10" s="12"/>
       <c r="M10" s="12"/>
@@ -1363,7 +1363,7 @@
       <c r="A13" s="2"/>
       <c r="B13" s="7"/>
       <c r="C13" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
@@ -1373,7 +1373,7 @@
       <c r="I13" s="9"/>
       <c r="J13" s="9"/>
       <c r="K13" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L13" s="9"/>
       <c r="M13" s="9"/>
@@ -1388,7 +1388,7 @@
       <c r="A14" s="2"/>
       <c r="B14" s="7"/>
       <c r="C14" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
@@ -1411,7 +1411,7 @@
       <c r="A15" s="2"/>
       <c r="B15" s="7"/>
       <c r="C15" s="19" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
@@ -1454,7 +1454,7 @@
     <row r="17" spans="2:19" ht="18">
       <c r="B17" s="7"/>
       <c r="C17" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
@@ -1499,14 +1499,14 @@
     <row r="19" spans="2:19" ht="18">
       <c r="B19" s="7"/>
       <c r="C19" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
       <c r="G19" s="54"/>
       <c r="H19" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I19" s="11"/>
       <c r="J19" s="9"/>
@@ -1525,14 +1525,14 @@
     <row r="20" spans="2:19" ht="18">
       <c r="B20" s="7"/>
       <c r="C20" s="55" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
       <c r="H20" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I20" s="9"/>
       <c r="J20" s="9"/>
@@ -1569,11 +1569,11 @@
     </row>
     <row r="22" spans="2:19" ht="34.25" customHeight="1">
       <c r="B22" s="7"/>
-      <c r="C22" s="73"/>
-      <c r="D22" s="73"/>
-      <c r="E22" s="73"/>
-      <c r="F22" s="73"/>
-      <c r="G22" s="73"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
+      <c r="E22" s="64"/>
+      <c r="F22" s="64"/>
+      <c r="G22" s="64"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="9"/>
@@ -1630,11 +1630,11 @@
     <row r="25" spans="2:19" ht="18">
       <c r="B25" s="7"/>
       <c r="C25" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -1656,11 +1656,11 @@
     <row r="26" spans="2:19" ht="18">
       <c r="B26" s="7"/>
       <c r="C26" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -1701,33 +1701,33 @@
     </row>
     <row r="28" spans="2:19" ht="21" customHeight="1">
       <c r="B28" s="7"/>
-      <c r="C28" s="64" t="s">
+      <c r="C28" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="D28" s="64"/>
-      <c r="E28" s="64"/>
-      <c r="F28" s="70" t="s">
+      <c r="D28" s="60"/>
+      <c r="E28" s="60"/>
+      <c r="F28" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="G28" s="70" t="s">
+      <c r="G28" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="H28" s="64" t="s">
+      <c r="H28" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="I28" s="64"/>
-      <c r="J28" s="64" t="s">
+      <c r="I28" s="60"/>
+      <c r="J28" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="K28" s="64"/>
-      <c r="L28" s="64" t="s">
+      <c r="K28" s="60"/>
+      <c r="L28" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="M28" s="71"/>
-      <c r="N28" s="71" t="s">
+      <c r="M28" s="62"/>
+      <c r="N28" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="O28" s="72"/>
+      <c r="O28" s="63"/>
       <c r="P28" s="10"/>
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
@@ -1735,11 +1735,11 @@
     </row>
     <row r="29" spans="2:19" ht="18">
       <c r="B29" s="7"/>
-      <c r="C29" s="64"/>
-      <c r="D29" s="64"/>
-      <c r="E29" s="64"/>
-      <c r="F29" s="70"/>
-      <c r="G29" s="70"/>
+      <c r="C29" s="60"/>
+      <c r="D29" s="60"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="61"/>
+      <c r="G29" s="61"/>
       <c r="H29" s="22" t="s">
         <v>14</v>
       </c>
@@ -1791,13 +1791,13 @@
     </row>
     <row r="31" spans="2:19" ht="99.9" customHeight="1">
       <c r="B31" s="7"/>
-      <c r="C31" s="61" t="s">
-        <v>52</v>
-      </c>
-      <c r="D31" s="62"/>
-      <c r="E31" s="63"/>
+      <c r="C31" s="69" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="70"/>
+      <c r="E31" s="71"/>
       <c r="F31" s="29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G31" s="30">
         <f>20028.63*51.68124</f>
@@ -1934,12 +1934,12 @@
     </row>
     <row r="37" spans="2:19" ht="18">
       <c r="B37" s="7"/>
-      <c r="C37" s="64" t="s">
+      <c r="C37" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="D37" s="64"/>
-      <c r="E37" s="64"/>
-      <c r="F37" s="64"/>
+      <c r="D37" s="60"/>
+      <c r="E37" s="60"/>
+      <c r="F37" s="60"/>
       <c r="G37" s="39">
         <f>SUM(G30:G36)</f>
         <v>1035104.4339012001</v>
@@ -2065,14 +2065,14 @@
       <c r="E42" s="9"/>
       <c r="F42" s="11"/>
       <c r="G42" s="9"/>
-      <c r="H42" s="65"/>
-      <c r="I42" s="66"/>
-      <c r="J42" s="65"/>
-      <c r="K42" s="66"/>
-      <c r="L42" s="65"/>
-      <c r="M42" s="67"/>
-      <c r="N42" s="65"/>
-      <c r="O42" s="66"/>
+      <c r="H42" s="72"/>
+      <c r="I42" s="73"/>
+      <c r="J42" s="72"/>
+      <c r="K42" s="73"/>
+      <c r="L42" s="72"/>
+      <c r="M42" s="74"/>
+      <c r="N42" s="72"/>
+      <c r="O42" s="73"/>
       <c r="P42" s="10"/>
       <c r="Q42" s="2"/>
       <c r="R42" s="2"/>
@@ -2132,7 +2132,7 @@
       <c r="J45" s="9"/>
       <c r="K45" s="9"/>
       <c r="L45" s="45" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M45" s="45"/>
       <c r="N45" s="9"/>
@@ -2145,7 +2145,7 @@
     <row r="46" spans="2:19" ht="18">
       <c r="B46" s="7"/>
       <c r="C46" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9"/>
@@ -2167,7 +2167,7 @@
     <row r="47" spans="2:19" ht="18">
       <c r="B47" s="7"/>
       <c r="C47" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
@@ -2189,7 +2189,7 @@
     <row r="48" spans="2:19" ht="18">
       <c r="B48" s="7"/>
       <c r="C48" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9"/>
@@ -2210,7 +2210,7 @@
     <row r="49" spans="2:19" ht="18">
       <c r="B49" s="7"/>
       <c r="C49" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
@@ -2231,7 +2231,7 @@
     <row r="50" spans="2:19" ht="18">
       <c r="B50" s="7"/>
       <c r="C50" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
@@ -2310,59 +2310,59 @@
     </row>
     <row r="54" spans="2:19" ht="15" customHeight="1">
       <c r="B54" s="7"/>
-      <c r="C54" s="58" t="s">
-        <v>36</v>
-      </c>
-      <c r="D54" s="58"/>
-      <c r="E54" s="58"/>
-      <c r="F54" s="58"/>
-      <c r="G54" s="58"/>
-      <c r="H54" s="58"/>
-      <c r="I54" s="58"/>
-      <c r="J54" s="58"/>
-      <c r="K54" s="58"/>
-      <c r="L54" s="58"/>
-      <c r="M54" s="58"/>
-      <c r="N54" s="58"/>
-      <c r="O54" s="58"/>
+      <c r="C54" s="66" t="s">
+        <v>35</v>
+      </c>
+      <c r="D54" s="66"/>
+      <c r="E54" s="66"/>
+      <c r="F54" s="66"/>
+      <c r="G54" s="66"/>
+      <c r="H54" s="66"/>
+      <c r="I54" s="66"/>
+      <c r="J54" s="66"/>
+      <c r="K54" s="66"/>
+      <c r="L54" s="66"/>
+      <c r="M54" s="66"/>
+      <c r="N54" s="66"/>
+      <c r="O54" s="66"/>
       <c r="P54" s="10"/>
       <c r="Q54" s="2"/>
       <c r="R54" s="2"/>
     </row>
     <row r="55" spans="2:19" ht="18">
       <c r="B55" s="7"/>
-      <c r="C55" s="58"/>
-      <c r="D55" s="58"/>
-      <c r="E55" s="58"/>
-      <c r="F55" s="58"/>
-      <c r="G55" s="58"/>
-      <c r="H55" s="58"/>
-      <c r="I55" s="58"/>
-      <c r="J55" s="58"/>
-      <c r="K55" s="58"/>
-      <c r="L55" s="58"/>
-      <c r="M55" s="58"/>
-      <c r="N55" s="58"/>
-      <c r="O55" s="58"/>
+      <c r="C55" s="66"/>
+      <c r="D55" s="66"/>
+      <c r="E55" s="66"/>
+      <c r="F55" s="66"/>
+      <c r="G55" s="66"/>
+      <c r="H55" s="66"/>
+      <c r="I55" s="66"/>
+      <c r="J55" s="66"/>
+      <c r="K55" s="66"/>
+      <c r="L55" s="66"/>
+      <c r="M55" s="66"/>
+      <c r="N55" s="66"/>
+      <c r="O55" s="66"/>
       <c r="P55" s="10"/>
       <c r="Q55" s="2"/>
       <c r="R55" s="2"/>
     </row>
     <row r="56" spans="2:19" ht="18">
       <c r="B56" s="7"/>
-      <c r="C56" s="58"/>
-      <c r="D56" s="58"/>
-      <c r="E56" s="58"/>
-      <c r="F56" s="58"/>
-      <c r="G56" s="58"/>
-      <c r="H56" s="58"/>
-      <c r="I56" s="58"/>
-      <c r="J56" s="58"/>
-      <c r="K56" s="58"/>
-      <c r="L56" s="58"/>
-      <c r="M56" s="58"/>
-      <c r="N56" s="58"/>
-      <c r="O56" s="58"/>
+      <c r="C56" s="66"/>
+      <c r="D56" s="66"/>
+      <c r="E56" s="66"/>
+      <c r="F56" s="66"/>
+      <c r="G56" s="66"/>
+      <c r="H56" s="66"/>
+      <c r="I56" s="66"/>
+      <c r="J56" s="66"/>
+      <c r="K56" s="66"/>
+      <c r="L56" s="66"/>
+      <c r="M56" s="66"/>
+      <c r="N56" s="66"/>
+      <c r="O56" s="66"/>
       <c r="P56" s="10"/>
       <c r="Q56" s="2"/>
       <c r="R56" s="2"/>
@@ -2370,19 +2370,19 @@
     </row>
     <row r="57" spans="2:19" ht="18">
       <c r="B57" s="7"/>
-      <c r="C57" s="58"/>
-      <c r="D57" s="58"/>
-      <c r="E57" s="58"/>
-      <c r="F57" s="58"/>
-      <c r="G57" s="58"/>
-      <c r="H57" s="58"/>
-      <c r="I57" s="58"/>
-      <c r="J57" s="58"/>
-      <c r="K57" s="58"/>
-      <c r="L57" s="58"/>
-      <c r="M57" s="58"/>
-      <c r="N57" s="58"/>
-      <c r="O57" s="58"/>
+      <c r="C57" s="66"/>
+      <c r="D57" s="66"/>
+      <c r="E57" s="66"/>
+      <c r="F57" s="66"/>
+      <c r="G57" s="66"/>
+      <c r="H57" s="66"/>
+      <c r="I57" s="66"/>
+      <c r="J57" s="66"/>
+      <c r="K57" s="66"/>
+      <c r="L57" s="66"/>
+      <c r="M57" s="66"/>
+      <c r="N57" s="66"/>
+      <c r="O57" s="66"/>
       <c r="P57" s="10"/>
       <c r="Q57" s="2"/>
       <c r="R57" s="2"/>
@@ -2390,19 +2390,19 @@
     </row>
     <row r="58" spans="2:19" ht="23.25" customHeight="1">
       <c r="B58" s="7"/>
-      <c r="C58" s="58"/>
-      <c r="D58" s="58"/>
-      <c r="E58" s="58"/>
-      <c r="F58" s="58"/>
-      <c r="G58" s="58"/>
-      <c r="H58" s="58"/>
-      <c r="I58" s="58"/>
-      <c r="J58" s="58"/>
-      <c r="K58" s="58"/>
-      <c r="L58" s="58"/>
-      <c r="M58" s="58"/>
-      <c r="N58" s="58"/>
-      <c r="O58" s="58"/>
+      <c r="C58" s="66"/>
+      <c r="D58" s="66"/>
+      <c r="E58" s="66"/>
+      <c r="F58" s="66"/>
+      <c r="G58" s="66"/>
+      <c r="H58" s="66"/>
+      <c r="I58" s="66"/>
+      <c r="J58" s="66"/>
+      <c r="K58" s="66"/>
+      <c r="L58" s="66"/>
+      <c r="M58" s="66"/>
+      <c r="N58" s="66"/>
+      <c r="O58" s="66"/>
       <c r="P58" s="10"/>
       <c r="Q58" s="2"/>
       <c r="R58" s="2"/>
@@ -2410,19 +2410,19 @@
     </row>
     <row r="59" spans="2:19" ht="23.25" customHeight="1">
       <c r="B59" s="7"/>
-      <c r="C59" s="58"/>
-      <c r="D59" s="58"/>
-      <c r="E59" s="58"/>
-      <c r="F59" s="58"/>
-      <c r="G59" s="58"/>
-      <c r="H59" s="58"/>
-      <c r="I59" s="58"/>
-      <c r="J59" s="58"/>
-      <c r="K59" s="58"/>
-      <c r="L59" s="58"/>
-      <c r="M59" s="58"/>
-      <c r="N59" s="58"/>
-      <c r="O59" s="58"/>
+      <c r="C59" s="66"/>
+      <c r="D59" s="66"/>
+      <c r="E59" s="66"/>
+      <c r="F59" s="66"/>
+      <c r="G59" s="66"/>
+      <c r="H59" s="66"/>
+      <c r="I59" s="66"/>
+      <c r="J59" s="66"/>
+      <c r="K59" s="66"/>
+      <c r="L59" s="66"/>
+      <c r="M59" s="66"/>
+      <c r="N59" s="66"/>
+      <c r="O59" s="66"/>
       <c r="P59" s="10"/>
       <c r="Q59" s="2"/>
       <c r="R59" s="2"/>
@@ -2430,19 +2430,19 @@
     </row>
     <row r="60" spans="2:19" ht="23.25" customHeight="1">
       <c r="B60" s="7"/>
-      <c r="C60" s="58"/>
-      <c r="D60" s="58"/>
-      <c r="E60" s="58"/>
-      <c r="F60" s="58"/>
-      <c r="G60" s="58"/>
-      <c r="H60" s="58"/>
-      <c r="I60" s="58"/>
-      <c r="J60" s="58"/>
-      <c r="K60" s="58"/>
-      <c r="L60" s="58"/>
-      <c r="M60" s="58"/>
-      <c r="N60" s="58"/>
-      <c r="O60" s="58"/>
+      <c r="C60" s="66"/>
+      <c r="D60" s="66"/>
+      <c r="E60" s="66"/>
+      <c r="F60" s="66"/>
+      <c r="G60" s="66"/>
+      <c r="H60" s="66"/>
+      <c r="I60" s="66"/>
+      <c r="J60" s="66"/>
+      <c r="K60" s="66"/>
+      <c r="L60" s="66"/>
+      <c r="M60" s="66"/>
+      <c r="N60" s="66"/>
+      <c r="O60" s="66"/>
       <c r="P60" s="10"/>
       <c r="Q60" s="2"/>
       <c r="R60" s="2"/>
@@ -2450,19 +2450,19 @@
     </row>
     <row r="61" spans="2:19" ht="23.25" customHeight="1">
       <c r="B61" s="7"/>
-      <c r="C61" s="58"/>
-      <c r="D61" s="58"/>
-      <c r="E61" s="58"/>
-      <c r="F61" s="58"/>
-      <c r="G61" s="58"/>
-      <c r="H61" s="58"/>
-      <c r="I61" s="58"/>
-      <c r="J61" s="58"/>
-      <c r="K61" s="58"/>
-      <c r="L61" s="58"/>
-      <c r="M61" s="58"/>
-      <c r="N61" s="58"/>
-      <c r="O61" s="58"/>
+      <c r="C61" s="66"/>
+      <c r="D61" s="66"/>
+      <c r="E61" s="66"/>
+      <c r="F61" s="66"/>
+      <c r="G61" s="66"/>
+      <c r="H61" s="66"/>
+      <c r="I61" s="66"/>
+      <c r="J61" s="66"/>
+      <c r="K61" s="66"/>
+      <c r="L61" s="66"/>
+      <c r="M61" s="66"/>
+      <c r="N61" s="66"/>
+      <c r="O61" s="66"/>
       <c r="P61" s="10"/>
       <c r="Q61" s="2"/>
       <c r="R61" s="2"/>
@@ -2510,21 +2510,21 @@
     </row>
     <row r="64" spans="2:19" ht="18" hidden="1">
       <c r="B64" s="7"/>
-      <c r="C64" s="59" t="s">
+      <c r="C64" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="D64" s="59"/>
-      <c r="E64" s="59"/>
-      <c r="F64" s="59"/>
-      <c r="G64" s="59"/>
-      <c r="H64" s="59"/>
-      <c r="I64" s="59"/>
-      <c r="J64" s="59"/>
-      <c r="K64" s="59"/>
-      <c r="L64" s="59"/>
-      <c r="M64" s="59"/>
-      <c r="N64" s="59"/>
-      <c r="O64" s="59"/>
+      <c r="D64" s="67"/>
+      <c r="E64" s="67"/>
+      <c r="F64" s="67"/>
+      <c r="G64" s="67"/>
+      <c r="H64" s="67"/>
+      <c r="I64" s="67"/>
+      <c r="J64" s="67"/>
+      <c r="K64" s="67"/>
+      <c r="L64" s="67"/>
+      <c r="M64" s="67"/>
+      <c r="N64" s="67"/>
+      <c r="O64" s="67"/>
       <c r="P64" s="10"/>
       <c r="Q64" s="2"/>
       <c r="R64" s="2"/>
@@ -2532,21 +2532,21 @@
     </row>
     <row r="65" spans="2:19" ht="18" hidden="1">
       <c r="B65" s="7"/>
-      <c r="C65" s="60" t="s">
+      <c r="C65" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="D65" s="60"/>
-      <c r="E65" s="60"/>
-      <c r="F65" s="60"/>
-      <c r="G65" s="60"/>
-      <c r="H65" s="60"/>
-      <c r="I65" s="60"/>
-      <c r="J65" s="60"/>
-      <c r="K65" s="60"/>
-      <c r="L65" s="60"/>
-      <c r="M65" s="60"/>
-      <c r="N65" s="60"/>
-      <c r="O65" s="60"/>
+      <c r="D65" s="68"/>
+      <c r="E65" s="68"/>
+      <c r="F65" s="68"/>
+      <c r="G65" s="68"/>
+      <c r="H65" s="68"/>
+      <c r="I65" s="68"/>
+      <c r="J65" s="68"/>
+      <c r="K65" s="68"/>
+      <c r="L65" s="68"/>
+      <c r="M65" s="68"/>
+      <c r="N65" s="68"/>
+      <c r="O65" s="68"/>
       <c r="P65" s="10"/>
       <c r="Q65" s="2"/>
       <c r="R65" s="2"/>
@@ -2574,6 +2574,16 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C54:O61"/>
+    <mergeCell ref="C64:O64"/>
+    <mergeCell ref="C65:O65"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="G40:O40"/>
     <mergeCell ref="B1:P1"/>
     <mergeCell ref="J4:M4"/>
     <mergeCell ref="J5:M5"/>
@@ -2586,16 +2596,6 @@
     <mergeCell ref="N28:O28"/>
     <mergeCell ref="C22:G22"/>
     <mergeCell ref="H7:J7"/>
-    <mergeCell ref="C54:O61"/>
-    <mergeCell ref="C64:O64"/>
-    <mergeCell ref="C65:O65"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="G40:O40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="55" orientation="portrait" r:id="rId1"/>

</xml_diff>